<commit_message>
Added outstanding 4116 and 4164 spreadsheets and updated config and hard coded timings based on assorted datasheets. Saved these datasheets to the timings directory. Converted 4116 to use generic 1b1r pio file and related mem_chip.c functions.
</commit_message>
<xml_diff>
--- a/firmware/timings/4116-120.xlsx
+++ b/firmware/timings/4116-120.xlsx
@@ -287,7 +287,7 @@
     <t>Blank the State Machine's Output Shift Register.</t>
   </si>
   <si>
-    <t>tCPN</t>
+    <t>tCP[N]</t>
   </si>
   <si>
     <t>nop [4]</t>
@@ -728,7 +728,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -830,6 +830,9 @@
     <xf borderId="3" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="6" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -852,7 +855,7 @@
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -5249,7 +5252,7 @@
       </c>
       <c r="K4" s="28">
         <f>J4+(OFFSET($B$4,$I4,0)+1)*cmd_time</f>
-        <v>123.3321</v>
+        <v>19.9998</v>
       </c>
       <c r="L4" s="26" t="s">
         <v>18</v>
@@ -5260,7 +5263,7 @@
         <v>1.0</v>
       </c>
       <c r="B5" s="23">
-        <v>31.0</v>
+        <v>0.0</v>
       </c>
       <c r="C5" s="24"/>
       <c r="D5" s="24"/>
@@ -5275,11 +5278,11 @@
       </c>
       <c r="J5" s="27">
         <f t="shared" ref="J5:J12" si="1">K4</f>
-        <v>123.3321</v>
+        <v>19.9998</v>
       </c>
       <c r="K5" s="28">
         <f>J5+(OFFSET($B$4,$I5,0)+1)*cmd_time</f>
-        <v>196.6647</v>
+        <v>86.6658</v>
       </c>
       <c r="L5" s="26" t="s">
         <v>20</v>
@@ -5290,7 +5293,7 @@
         <v>2.0</v>
       </c>
       <c r="B6" s="23">
-        <v>21.0</v>
+        <v>19.0</v>
       </c>
       <c r="C6" s="24"/>
       <c r="D6" s="24"/>
@@ -5305,11 +5308,11 @@
       </c>
       <c r="J6" s="27">
         <f t="shared" si="1"/>
-        <v>196.6647</v>
+        <v>86.6658</v>
       </c>
       <c r="K6" s="28">
         <f>J6+(OFFSET($B$4,$I6,0)+1)*cmd_time</f>
-        <v>199.998</v>
+        <v>89.9991</v>
       </c>
       <c r="L6" s="26" t="s">
         <v>22</v>
@@ -5320,7 +5323,7 @@
         <v>3.0</v>
       </c>
       <c r="B7" s="23">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="C7" s="24"/>
       <c r="D7" s="24"/>
@@ -5335,11 +5338,11 @@
       </c>
       <c r="J7" s="27">
         <f t="shared" si="1"/>
-        <v>199.998</v>
+        <v>89.9991</v>
       </c>
       <c r="K7" s="28">
         <f>J7+(OFFSET($B$4,$I7,0)+1)*cmd_time</f>
-        <v>203.3313</v>
+        <v>93.3324</v>
       </c>
       <c r="L7" s="26" t="s">
         <v>24</v>
@@ -5350,7 +5353,7 @@
         <v>4.0</v>
       </c>
       <c r="B8" s="23">
-        <v>8.0</v>
+        <v>12.0</v>
       </c>
       <c r="C8" s="24"/>
       <c r="D8" s="24"/>
@@ -5365,11 +5368,11 @@
       </c>
       <c r="J8" s="27">
         <f t="shared" si="1"/>
-        <v>203.3313</v>
+        <v>93.3324</v>
       </c>
       <c r="K8" s="28">
         <f>J8+(OFFSET($B$4,$I8,0)+1)*cmd_time</f>
-        <v>209.9979</v>
+        <v>106.6656</v>
       </c>
       <c r="L8" s="26" t="s">
         <v>26</v>
@@ -5380,7 +5383,7 @@
         <v>5.0</v>
       </c>
       <c r="B9" s="23">
-        <v>9.0</v>
+        <v>8.0</v>
       </c>
       <c r="C9" s="24"/>
       <c r="D9" s="24"/>
@@ -5397,11 +5400,11 @@
       </c>
       <c r="J9" s="27">
         <f t="shared" si="1"/>
-        <v>209.9979</v>
+        <v>106.6656</v>
       </c>
       <c r="K9" s="28">
         <f>J9+(OFFSET($B$4,$I9,0)+1)*cmd_time</f>
-        <v>213.3312</v>
+        <v>109.9989</v>
       </c>
       <c r="L9" s="26" t="s">
         <v>29</v>
@@ -5412,7 +5415,7 @@
         <v>6.0</v>
       </c>
       <c r="B10" s="23">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
@@ -5427,11 +5430,11 @@
       </c>
       <c r="J10" s="27">
         <f t="shared" si="1"/>
-        <v>213.3312</v>
+        <v>109.9989</v>
       </c>
       <c r="K10" s="28">
         <f>J10+(OFFSET($B$4,$I10,0)+1)*cmd_time</f>
-        <v>216.6645</v>
+        <v>113.3322</v>
       </c>
       <c r="L10" s="26" t="s">
         <v>31</v>
@@ -5442,7 +5445,7 @@
         <v>7.0</v>
       </c>
       <c r="B11" s="23">
-        <v>8.0</v>
+        <v>0.0</v>
       </c>
       <c r="C11" s="24"/>
       <c r="D11" s="24"/>
@@ -5457,11 +5460,11 @@
       </c>
       <c r="J11" s="30">
         <f t="shared" si="1"/>
-        <v>216.6645</v>
+        <v>113.3322</v>
       </c>
       <c r="K11" s="28">
         <f>J11+(OFFSET($B$4,$I11,0)+1)*cmd_time</f>
-        <v>219.9978</v>
+        <v>116.6655</v>
       </c>
       <c r="L11" s="26" t="s">
         <v>33</v>
@@ -5485,11 +5488,11 @@
       </c>
       <c r="J12" s="27">
         <f t="shared" si="1"/>
-        <v>219.9978</v>
+        <v>116.6655</v>
       </c>
       <c r="K12" s="28">
         <f>J12+(OFFSET($B$4,$I12,0)+1)*cmd_time</f>
-        <v>223.3311</v>
+        <v>119.9988</v>
       </c>
       <c r="L12" s="26" t="s">
         <v>35</v>
@@ -5519,11 +5522,11 @@
       </c>
       <c r="J13" s="31">
         <f>K10</f>
-        <v>216.6645</v>
+        <v>113.3322</v>
       </c>
       <c r="K13" s="28">
         <f>J13+(OFFSET($B$4,$I13,0)+1)*cmd_time</f>
-        <v>219.9978</v>
+        <v>116.6655</v>
       </c>
       <c r="L13" s="26" t="s">
         <v>41</v>
@@ -5542,7 +5545,7 @@
       </c>
       <c r="D14" s="33">
         <f>ROUND(ras_low_start - ras_high_end,1)</f>
-        <v>196.7</v>
+        <v>86.7</v>
       </c>
       <c r="E14" s="19"/>
       <c r="F14" s="19"/>
@@ -5555,11 +5558,11 @@
       </c>
       <c r="J14" s="34">
         <f>K13</f>
-        <v>219.9978</v>
+        <v>116.6655</v>
       </c>
       <c r="K14" s="28">
         <f>J14+(OFFSET($B$4,$I14,0)+1)*cmd_time</f>
-        <v>223.3311</v>
+        <v>119.9988</v>
       </c>
       <c r="L14" s="26" t="s">
         <v>44</v>
@@ -5569,16 +5572,16 @@
       <c r="A15" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="25">
-        <v>15.0</v>
+      <c r="B15" s="23">
+        <v>10.0</v>
       </c>
       <c r="C15" s="32">
         <f>B15 + (B15 * tolerance/100)</f>
-        <v>13.5</v>
+        <v>9</v>
       </c>
       <c r="D15" s="33">
         <f>ROUND(asc_start - ras_low_end, 1)</f>
-        <v>6.7</v>
+        <v>13.3</v>
       </c>
       <c r="E15" s="19"/>
       <c r="F15" s="19"/>
@@ -5593,30 +5596,30 @@
       </c>
       <c r="J15" s="27">
         <f>K12</f>
-        <v>223.3311</v>
+        <v>119.9988</v>
       </c>
       <c r="K15" s="28">
         <f>J15+(OFFSET($B$4,$I15,0)+1)*cmd_time</f>
-        <v>226.6644</v>
+        <v>123.3321</v>
       </c>
       <c r="L15" s="26" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="29" t="s">
+      <c r="A16" s="35" t="s">
         <v>49</v>
       </c>
       <c r="B16" s="23">
-        <v>0.0</v>
+        <v>45.0</v>
       </c>
       <c r="C16" s="32">
         <f>B16 + (B16 * tolerance/100)</f>
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="D16" s="33">
         <f>ROUND(max(cas_low_start_w-cas_high_end,cas_low_start_r-cas_high_end),1)</f>
-        <v>213.3</v>
+        <v>110</v>
       </c>
       <c r="E16" s="19"/>
       <c r="F16" s="19"/>
@@ -5629,11 +5632,11 @@
       </c>
       <c r="J16" s="27">
         <f t="shared" ref="J16:J24" si="2">K15</f>
-        <v>226.6644</v>
+        <v>123.3321</v>
       </c>
       <c r="K16" s="28">
         <f>J16+(OFFSET($B$4,$I16,0)+1)*cmd_time</f>
-        <v>256.6641</v>
+        <v>166.665</v>
       </c>
       <c r="L16" s="26" t="s">
         <v>51</v>
@@ -5643,7 +5646,7 @@
       <c r="A17" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="23">
         <v>15.0</v>
       </c>
       <c r="C17" s="32">
@@ -5652,7 +5655,7 @@
       </c>
       <c r="D17" s="33">
         <f>ROUND(cas_low_start_w - ras_low_end,1)</f>
-        <v>13.3</v>
+        <v>20</v>
       </c>
       <c r="E17" s="19"/>
       <c r="F17" s="19"/>
@@ -5665,11 +5668,11 @@
       </c>
       <c r="J17" s="27">
         <f t="shared" si="2"/>
-        <v>256.6641</v>
+        <v>166.665</v>
       </c>
       <c r="K17" s="28">
         <f>J17+(OFFSET($B$4,$I17,0)+1)*cmd_time</f>
-        <v>259.9974</v>
+        <v>169.9983</v>
       </c>
       <c r="L17" s="26" t="s">
         <v>53</v>
@@ -5688,7 +5691,7 @@
       </c>
       <c r="D18" s="33">
         <f>ROUND(cas_low_start_w - ras_low_end,1)</f>
-        <v>13.3</v>
+        <v>20</v>
       </c>
       <c r="E18" s="19"/>
       <c r="F18" s="19"/>
@@ -5701,11 +5704,11 @@
       </c>
       <c r="J18" s="27">
         <f t="shared" si="2"/>
-        <v>259.9974</v>
+        <v>169.9983</v>
       </c>
       <c r="K18" s="28">
         <f>J18+(OFFSET($B$4,$I18,0)+1)*cmd_time</f>
-        <v>263.3307</v>
+        <v>173.3316</v>
       </c>
       <c r="L18" s="26" t="s">
         <v>55</v>
@@ -5715,16 +5718,16 @@
       <c r="A19" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="35">
-        <v>40.0</v>
+      <c r="B19" s="36">
+        <v>25.0</v>
       </c>
       <c r="C19" s="32">
         <f>B19 + (B19 * tolerance/100)</f>
-        <v>36</v>
+        <v>22.5</v>
       </c>
       <c r="D19" s="33">
         <f>ROUND(w_high_start_2 - cas_low_end_w, 1)</f>
-        <v>36.7</v>
+        <v>50</v>
       </c>
       <c r="E19" s="19"/>
       <c r="F19" s="19"/>
@@ -5737,11 +5740,11 @@
       </c>
       <c r="J19" s="27">
         <f t="shared" si="2"/>
-        <v>263.3307</v>
+        <v>173.3316</v>
       </c>
       <c r="K19" s="28">
         <f>J19+(OFFSET($B$4,$I19,0)+1)*cmd_time</f>
-        <v>296.6637</v>
+        <v>203.3313</v>
       </c>
       <c r="L19" s="26" t="s">
         <v>58</v>
@@ -5752,15 +5755,15 @@
         <v>59</v>
       </c>
       <c r="B20" s="23">
-        <v>40.0</v>
+        <v>25.0</v>
       </c>
       <c r="C20" s="32">
         <f>B20 + (B20 * tolerance/100)</f>
-        <v>36</v>
+        <v>22.5</v>
       </c>
       <c r="D20" s="33">
         <f>ROUND(w_high_start_2 - w_low_end, 1)</f>
-        <v>36.7</v>
+        <v>50</v>
       </c>
       <c r="E20" s="19"/>
       <c r="F20" s="19"/>
@@ -5773,11 +5776,11 @@
       </c>
       <c r="J20" s="27">
         <f t="shared" si="2"/>
-        <v>296.6637</v>
+        <v>203.3313</v>
       </c>
       <c r="K20" s="28">
         <f>J20+(OFFSET($B$4,$I20,0)+1)*cmd_time</f>
-        <v>299.997</v>
+        <v>206.6646</v>
       </c>
       <c r="L20" s="26" t="s">
         <v>61</v>
@@ -5796,7 +5799,7 @@
       </c>
       <c r="D21" s="33">
         <f>ROUND(w_high_start_2 - ras_low_end, 1)</f>
-        <v>53.3</v>
+        <v>73.3</v>
       </c>
       <c r="E21" s="19"/>
       <c r="F21" s="19"/>
@@ -5809,11 +5812,11 @@
       </c>
       <c r="J21" s="27">
         <f t="shared" si="2"/>
-        <v>299.997</v>
+        <v>206.6646</v>
       </c>
       <c r="K21" s="28">
         <f>J21+(OFFSET($B$4,$I21,0)+1)*cmd_time</f>
-        <v>303.3303</v>
+        <v>209.9979</v>
       </c>
       <c r="L21" s="26" t="s">
         <v>63</v>
@@ -5824,15 +5827,15 @@
         <v>64</v>
       </c>
       <c r="B22" s="23">
-        <v>40.0</v>
+        <v>15.0</v>
       </c>
       <c r="C22" s="32">
         <f>B22 + (B22 * tolerance/100)</f>
-        <v>36</v>
+        <v>13.5</v>
       </c>
       <c r="D22" s="33">
         <f>ROUND(col_clear_start - cas_low_end_w, 1)</f>
-        <v>40</v>
+        <v>53.3</v>
       </c>
       <c r="E22" s="19"/>
       <c r="F22" s="19"/>
@@ -5845,11 +5848,11 @@
       </c>
       <c r="J22" s="27">
         <f t="shared" si="2"/>
-        <v>303.3303</v>
+        <v>209.9979</v>
       </c>
       <c r="K22" s="28">
         <f>J22+(OFFSET($B$4,$I22,0)+1)*cmd_time</f>
-        <v>306.6636</v>
+        <v>213.3312</v>
       </c>
       <c r="L22" s="26"/>
     </row>
@@ -5864,9 +5867,9 @@
         <f>B23 + (B23 * tolerance/100)</f>
         <v>72</v>
       </c>
-      <c r="D23" s="36">
+      <c r="D23" s="37">
         <f>round(d_clear_start - ras_low_end, 1)</f>
-        <v>56.7</v>
+        <v>76.7</v>
       </c>
       <c r="E23" s="19"/>
       <c r="F23" s="19"/>
@@ -5879,11 +5882,11 @@
       </c>
       <c r="J23" s="27">
         <f t="shared" si="2"/>
-        <v>306.6636</v>
+        <v>213.3312</v>
       </c>
       <c r="K23" s="28">
         <f>J23+(OFFSET($B$4,$I23,0)+1)*cmd_time</f>
-        <v>319.9968</v>
+        <v>216.6645</v>
       </c>
       <c r="L23" s="26" t="s">
         <v>68</v>
@@ -5902,7 +5905,7 @@
       </c>
       <c r="D24" s="33">
         <f>ROUND(valid_data_start -ras_low_end, 1)</f>
-        <v>93.3</v>
+        <v>110</v>
       </c>
       <c r="E24" s="19"/>
       <c r="F24" s="19"/>
@@ -5915,13 +5918,13 @@
       </c>
       <c r="J24" s="27">
         <f t="shared" si="2"/>
-        <v>319.9968</v>
+        <v>216.6645</v>
       </c>
       <c r="K24" s="28">
         <f>J24+(OFFSET($B$4,$I24,0)+1)*cmd_time</f>
-        <v>323.3301</v>
-      </c>
-      <c r="L24" s="37" t="s">
+        <v>219.9978</v>
+      </c>
+      <c r="L24" s="38" t="s">
         <v>71</v>
       </c>
     </row>
@@ -5930,15 +5933,15 @@
         <v>72</v>
       </c>
       <c r="B25" s="23">
-        <v>80.0</v>
+        <v>60.0</v>
       </c>
       <c r="C25" s="32">
         <f>B25 + (B25 * tolerance/100)</f>
-        <v>72</v>
+        <v>54</v>
       </c>
       <c r="D25" s="33">
         <f>ROUND(cas_high_start - cas_low_end_w, 1)</f>
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="E25" s="19"/>
       <c r="F25" s="19"/>
@@ -5949,10 +5952,10 @@
       <c r="I25" s="26">
         <v>0.0</v>
       </c>
-      <c r="J25" s="38">
+      <c r="J25" s="39">
         <v>0.0</v>
       </c>
-      <c r="K25" s="39">
+      <c r="K25" s="40">
         <f>J25+cmd_time</f>
         <v>3.3333</v>
       </c>
@@ -5971,7 +5974,7 @@
       </c>
       <c r="D26" s="33">
         <f>ROUND(cas_high_start - ras_low_end,1)</f>
-        <v>96.7</v>
+        <v>113.3</v>
       </c>
       <c r="E26" s="19"/>
       <c r="F26" s="19"/>
@@ -6008,7 +6011,7 @@
       </c>
       <c r="D27" s="33">
         <f>round(cas_high_start - w_low_end, 1)</f>
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="E27" s="19"/>
       <c r="F27" s="19"/>
@@ -6044,7 +6047,7 @@
       </c>
       <c r="D28" s="33">
         <f>ROUND(ras_high_start - ras_low_end, 1)</f>
-        <v>120</v>
+        <v>126.7</v>
       </c>
       <c r="E28" s="19"/>
       <c r="F28" s="19"/>
@@ -6070,15 +6073,15 @@
         <v>83</v>
       </c>
       <c r="B29" s="23">
-        <v>320.0</v>
+        <v>230.0</v>
       </c>
       <c r="C29" s="32">
         <f>B29 + (B29 * tolerance/100)</f>
-        <v>288</v>
+        <v>207</v>
       </c>
       <c r="D29" s="33">
         <f>ras_high_start</f>
-        <v>323.3301</v>
+        <v>219.9978</v>
       </c>
       <c r="E29" s="19"/>
       <c r="F29" s="19"/>
@@ -6106,11 +6109,11 @@
       <c r="B30" s="23">
         <v>50.0</v>
       </c>
-      <c r="C30" s="40">
+      <c r="C30" s="41">
         <f>B30 + (B30 * tolerance/100)</f>
         <v>45</v>
       </c>
-      <c r="D30" s="41">
+      <c r="D30" s="42">
         <f>round(ras_high_start - w_low_end, 1)</f>
         <v>103.3</v>
       </c>
@@ -6137,11 +6140,11 @@
       <c r="A31" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="B31" s="42">
+      <c r="B31" s="43">
         <v>-10.0</v>
       </c>
-      <c r="C31" s="43"/>
-      <c r="D31" s="44"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="45"/>
       <c r="E31" s="24"/>
       <c r="F31" s="24"/>
       <c r="G31" s="25"/>
@@ -6151,7 +6154,7 @@
       <c r="I31" s="26">
         <v>7.0</v>
       </c>
-      <c r="J31" s="45"/>
+      <c r="J31" s="46"/>
       <c r="K31" s="26"/>
       <c r="L31" s="26" t="s">
         <v>89</v>
@@ -6171,17 +6174,17 @@
       <c r="I32" s="26">
         <v>0.0</v>
       </c>
-      <c r="J32" s="45"/>
+      <c r="J32" s="46"/>
       <c r="K32" s="26"/>
       <c r="L32" s="26"/>
     </row>
     <row r="33">
-      <c r="A33" s="46" t="s">
+      <c r="A33" s="47" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="47"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="48"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="49"/>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
       <c r="G33" s="7"/>

</xml_diff>